<commit_message>
thay đổi file esp
</commit_message>
<xml_diff>
--- a/Checklist_Project_Group_PRJ301_FA26.xlsx
+++ b/Checklist_Project_Group_PRJ301_FA26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FPT\learningProplem\PRJ\Project_Final\PRJ_SE2022_GR2_Project-final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9991055-B6C6-410D-BC32-129B78AE6528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC94C44-8C2F-47F0-9251-6C47F5AED907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="282">
   <si>
     <t>CHECKLIST PROJECT NHÓM PRJ301 FALL 2026</t>
   </si>
@@ -867,6 +867,9 @@
   </si>
   <si>
     <t>Đã soát xong trên tổng số</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -1341,7 +1344,9 @@
         <v>13</v>
       </c>
       <c r="G5" s="3"/>
-      <c r="H5" s="4"/>
+      <c r="H5" s="4" t="s">
+        <v>281</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3">

</xml_diff>

<commit_message>
sửa logout và quyền của device controler
</commit_message>
<xml_diff>
--- a/Checklist_Project_Group_PRJ301_FA26.xlsx
+++ b/Checklist_Project_Group_PRJ301_FA26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FPT\learningProplem\PRJ\Project_Final\PRJ_SE2022_GR2_Project-final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DC94C44-8C2F-47F0-9251-6C47F5AED907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B9F668E-1EE0-48A9-A3A7-D69F52BA4D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="287">
   <si>
     <t>CHECKLIST PROJECT NHÓM PRJ301 FALL 2026</t>
   </si>
@@ -870,6 +870,21 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>kiểm tra dữ liệu để chung với thêm dữ liệu mẫu</t>
+  </si>
+  <si>
+    <t>Xong</t>
+  </si>
+  <si>
+    <t>nhớ làm trên báo cáo</t>
+  </si>
+  <si>
+    <t>check lại sau khi hoàn thành toàn bộ</t>
+  </si>
+  <si>
+    <t>nhớ làm cái này</t>
   </si>
 </sst>
 </file>
@@ -991,6 +1006,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1002,14 +1025,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1254,7 +1269,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -1266,29 +1281,29 @@
     <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:8" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-    </row>
-    <row r="2" spans="1:8" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-    </row>
-    <row r="3" spans="1:8" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" spans="1:8" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+    </row>
+    <row r="3" spans="1:8" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1314,19 +1329,19 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-    </row>
-    <row r="5" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>1</v>
       </c>
@@ -1348,7 +1363,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>2</v>
       </c>
@@ -1368,7 +1383,7 @@
       <c r="G6" s="3"/>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>3</v>
       </c>
@@ -1385,10 +1400,14 @@
       <c r="F7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="G7" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>4</v>
       </c>
@@ -1405,10 +1424,12 @@
       <c r="F8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="3"/>
+      <c r="G8" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H8" s="4"/>
     </row>
-    <row r="9" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>5</v>
       </c>
@@ -1425,10 +1446,14 @@
       <c r="F9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="G9" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>6</v>
       </c>
@@ -1445,22 +1470,24 @@
       <c r="F10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="3"/>
+      <c r="G10" s="3" t="s">
+        <v>283</v>
+      </c>
       <c r="H10" s="4"/>
     </row>
-    <row r="11" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-    </row>
-    <row r="12" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+    </row>
+    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>7</v>
       </c>
@@ -1478,11 +1505,11 @@
         <v>33</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>34</v>
+        <v>283</v>
       </c>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>8</v>
       </c>
@@ -1500,11 +1527,11 @@
         <v>37</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>34</v>
+        <v>283</v>
       </c>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>9</v>
       </c>
@@ -1524,9 +1551,11 @@
       <c r="G14" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="H14" s="4" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>10</v>
       </c>
@@ -1544,11 +1573,13 @@
         <v>43</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>11</v>
       </c>
@@ -1570,7 +1601,7 @@
       </c>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>12</v>
       </c>
@@ -1588,23 +1619,23 @@
         <v>49</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>34</v>
+        <v>283</v>
       </c>
       <c r="H17" s="4"/>
     </row>
-    <row r="18" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-    </row>
-    <row r="19" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>13</v>
       </c>
@@ -1622,11 +1653,11 @@
         <v>54</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>34</v>
+        <v>283</v>
       </c>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>14</v>
       </c>
@@ -1648,7 +1679,7 @@
       </c>
       <c r="H20" s="4"/>
     </row>
-    <row r="21" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>15</v>
       </c>
@@ -1666,11 +1697,11 @@
         <v>60</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>34</v>
+        <v>283</v>
       </c>
       <c r="H21" s="4"/>
     </row>
-    <row r="22" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>16</v>
       </c>
@@ -1688,11 +1719,11 @@
         <v>63</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>34</v>
+        <v>283</v>
       </c>
       <c r="H22" s="4"/>
     </row>
-    <row r="23" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>17</v>
       </c>
@@ -1714,7 +1745,7 @@
       </c>
       <c r="H23" s="4"/>
     </row>
-    <row r="24" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>18</v>
       </c>
@@ -1736,7 +1767,7 @@
       </c>
       <c r="H24" s="4"/>
     </row>
-    <row r="25" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>19</v>
       </c>
@@ -1758,7 +1789,7 @@
       </c>
       <c r="H25" s="4"/>
     </row>
-    <row r="26" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>20</v>
       </c>
@@ -1780,19 +1811,19 @@
       </c>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>21</v>
       </c>
@@ -1812,7 +1843,7 @@
       <c r="G28" s="3"/>
       <c r="H28" s="4"/>
     </row>
-    <row r="29" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>22</v>
       </c>
@@ -1832,7 +1863,7 @@
       <c r="G29" s="3"/>
       <c r="H29" s="4"/>
     </row>
-    <row r="30" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>23</v>
       </c>
@@ -1852,7 +1883,7 @@
       <c r="G30" s="3"/>
       <c r="H30" s="4"/>
     </row>
-    <row r="31" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>24</v>
       </c>
@@ -1872,7 +1903,7 @@
       <c r="G31" s="3"/>
       <c r="H31" s="4"/>
     </row>
-    <row r="32" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>25</v>
       </c>
@@ -1892,7 +1923,7 @@
       <c r="G32" s="3"/>
       <c r="H32" s="4"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>26</v>
       </c>
@@ -1912,7 +1943,7 @@
       <c r="G33" s="3"/>
       <c r="H33" s="4"/>
     </row>
-    <row r="34" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>27</v>
       </c>
@@ -1932,19 +1963,19 @@
       <c r="G34" s="3"/>
       <c r="H34" s="4"/>
     </row>
-    <row r="35" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" s="13" t="s">
+      <c r="B35" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-    </row>
-    <row r="36" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+    </row>
+    <row r="36" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>28</v>
       </c>
@@ -1966,7 +1997,7 @@
       </c>
       <c r="H36" s="4"/>
     </row>
-    <row r="37" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>29</v>
       </c>
@@ -1988,7 +2019,7 @@
       </c>
       <c r="H37" s="4"/>
     </row>
-    <row r="38" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>30</v>
       </c>
@@ -2010,7 +2041,7 @@
       </c>
       <c r="H38" s="4"/>
     </row>
-    <row r="39" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>31</v>
       </c>
@@ -2032,19 +2063,19 @@
       </c>
       <c r="H39" s="4"/>
     </row>
-    <row r="40" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-    </row>
-    <row r="41" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+    </row>
+    <row r="41" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>32</v>
       </c>
@@ -2066,7 +2097,7 @@
       </c>
       <c r="H41" s="4"/>
     </row>
-    <row r="42" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>33</v>
       </c>
@@ -2088,7 +2119,7 @@
       </c>
       <c r="H42" s="4"/>
     </row>
-    <row r="43" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>34</v>
       </c>
@@ -2110,7 +2141,7 @@
       </c>
       <c r="H43" s="4"/>
     </row>
-    <row r="44" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>35</v>
       </c>
@@ -2132,7 +2163,7 @@
       </c>
       <c r="H44" s="4"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>36</v>
       </c>
@@ -2154,7 +2185,7 @@
       </c>
       <c r="H45" s="4"/>
     </row>
-    <row r="46" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>37</v>
       </c>
@@ -2176,15 +2207,15 @@
       </c>
       <c r="H46" s="4"/>
     </row>
-    <row r="47" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5"/>
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="C47" s="16"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
-      <c r="F47" s="16"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="11"/>
       <c r="G47" s="6"/>
       <c r="H47" s="5"/>
     </row>
@@ -2216,7 +2247,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2226,27 +2257,27 @@
     <col min="6" max="6" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-    </row>
-    <row r="2" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+    </row>
+    <row r="2" spans="1:6" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-    </row>
-    <row r="3" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+    </row>
+    <row r="3" spans="1:6" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>134</v>
       </c>
@@ -2266,7 +2297,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>140</v>
       </c>
@@ -2286,7 +2317,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>146</v>
       </c>
@@ -2304,7 +2335,7 @@
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>150</v>
       </c>
@@ -2322,7 +2353,7 @@
       </c>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>155</v>
       </c>
@@ -2340,7 +2371,7 @@
       </c>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>160</v>
       </c>
@@ -2358,25 +2389,25 @@
       </c>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" spans="1:6" ht="46.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:6" ht="46.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-    </row>
-    <row r="10" spans="1:6" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+    </row>
+    <row r="10" spans="1:6" ht="64.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2396,7 +2427,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E62"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -2405,23 +2436,23 @@
     <col min="5" max="5" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:5" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-    </row>
-    <row r="2" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-    </row>
-    <row r="3" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+    </row>
+    <row r="2" spans="1:5" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+    </row>
+    <row r="3" spans="1:5" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -2438,16 +2469,16 @@
         <v>171</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-    </row>
-    <row r="5" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+    </row>
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>1</v>
       </c>
@@ -2464,7 +2495,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>2</v>
       </c>
@@ -2481,7 +2512,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>3</v>
       </c>
@@ -2498,7 +2529,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>4</v>
       </c>
@@ -2515,7 +2546,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>5</v>
       </c>
@@ -2532,7 +2563,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>6</v>
       </c>
@@ -2549,16 +2580,16 @@
         <v>175</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-    </row>
-    <row r="12" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>7</v>
       </c>
@@ -2575,7 +2606,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>8</v>
       </c>
@@ -2592,7 +2623,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>9</v>
       </c>
@@ -2609,7 +2640,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>10</v>
       </c>
@@ -2626,7 +2657,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>11</v>
       </c>
@@ -2643,7 +2674,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>12</v>
       </c>
@@ -2660,16 +2691,16 @@
         <v>175</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-    </row>
-    <row r="19" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+    </row>
+    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>13</v>
       </c>
@@ -2686,7 +2717,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>14</v>
       </c>
@@ -2703,7 +2734,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>15</v>
       </c>
@@ -2720,7 +2751,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>16</v>
       </c>
@@ -2737,7 +2768,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>17</v>
       </c>
@@ -2754,7 +2785,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>18</v>
       </c>
@@ -2771,16 +2802,16 @@
         <v>175</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-    </row>
-    <row r="26" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+    </row>
+    <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>19</v>
       </c>
@@ -2797,7 +2828,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>20</v>
       </c>
@@ -2814,7 +2845,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>21</v>
       </c>
@@ -2831,7 +2862,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>22</v>
       </c>
@@ -2848,7 +2879,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>23</v>
       </c>
@@ -2865,7 +2896,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>24</v>
       </c>
@@ -2882,7 +2913,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>25</v>
       </c>
@@ -2899,7 +2930,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>26</v>
       </c>
@@ -2916,7 +2947,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>27</v>
       </c>
@@ -2933,16 +2964,16 @@
         <v>175</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" s="13" t="s">
+      <c r="B35" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>28</v>
       </c>
@@ -2959,7 +2990,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>29</v>
       </c>
@@ -2976,7 +3007,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>30</v>
       </c>
@@ -2993,7 +3024,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>31</v>
       </c>
@@ -3010,7 +3041,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>32</v>
       </c>
@@ -3027,7 +3058,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>33</v>
       </c>
@@ -3044,7 +3075,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>34</v>
       </c>
@@ -3061,16 +3092,16 @@
         <v>175</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
-      <c r="B43" s="13" t="s">
+      <c r="B43" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>35</v>
       </c>
@@ -3087,7 +3118,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>36</v>
       </c>
@@ -3104,7 +3135,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>37</v>
       </c>
@@ -3121,7 +3152,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>38</v>
       </c>
@@ -3138,7 +3169,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>39</v>
       </c>
@@ -3155,16 +3186,16 @@
         <v>175</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
-      <c r="B49" s="13" t="s">
+      <c r="B49" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>40</v>
       </c>
@@ -3181,7 +3212,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>41</v>
       </c>
@@ -3198,7 +3229,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>42</v>
       </c>
@@ -3215,7 +3246,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>43</v>
       </c>
@@ -3232,7 +3263,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>44</v>
       </c>
@@ -3249,16 +3280,16 @@
         <v>175</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
-      <c r="B55" s="13" t="s">
+      <c r="B55" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-    </row>
-    <row r="56" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+    </row>
+    <row r="56" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>45</v>
       </c>
@@ -3275,7 +3306,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>46</v>
       </c>
@@ -3292,7 +3323,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>47</v>
       </c>
@@ -3309,7 +3340,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>48</v>
       </c>
@@ -3326,7 +3357,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>49</v>
       </c>
@@ -3343,7 +3374,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>50</v>
       </c>
@@ -3360,13 +3391,13 @@
         <v>175</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5"/>
-      <c r="B62" s="15" t="s">
+      <c r="B62" s="10" t="s">
         <v>280</v>
       </c>
-      <c r="C62" s="16"/>
-      <c r="D62" s="16"/>
+      <c r="C62" s="11"/>
+      <c r="D62" s="11"/>
       <c r="E62" s="6"/>
     </row>
   </sheetData>

</xml_diff>